<commit_message>
today prac and lab 6 added
</commit_message>
<xml_diff>
--- a/practice.xlsx
+++ b/practice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e43f172441098b51/Desktop/Excel_first/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="8_{D3762795-6DE7-487B-9BAD-EEFD82822D72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BEEFE1FA-D7EE-4B04-B109-7BAF0E35D606}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="8_{D3762795-6DE7-487B-9BAD-EEFD82822D72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{023FBBC8-225C-418F-AC31-B7E50808137A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{E5A8AFDF-4C2B-4EF7-9F1C-64D71BC673BF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="54">
   <si>
     <t>Shashi</t>
   </si>
@@ -185,10 +185,19 @@
     <t>counta</t>
   </si>
   <si>
-    <t>hello</t>
-  </si>
-  <si>
     <t>countblank</t>
+  </si>
+  <si>
+    <t>Result</t>
+  </si>
+  <si>
+    <t>And</t>
+  </si>
+  <si>
+    <t>0r</t>
+  </si>
+  <si>
+    <t>if error</t>
   </si>
 </sst>
 </file>
@@ -239,19 +248,36 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="4">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -264,15 +290,30 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{56911E11-08A8-4610-9FE4-6E5B4F891A9E}" name="Table1" displayName="Table1" ref="C4:G14" totalsRowShown="0">
-  <autoFilter ref="C4:G14" xr:uid="{56911E11-08A8-4610-9FE4-6E5B4F891A9E}"/>
-  <tableColumns count="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{56911E11-08A8-4610-9FE4-6E5B4F891A9E}" name="Table1" displayName="Table1" ref="C4:J13" totalsRowShown="0">
+  <autoFilter ref="C4:J13" xr:uid="{56911E11-08A8-4610-9FE4-6E5B4F891A9E}"/>
+  <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{A6B0653E-CA82-4432-A5F6-E15402ED067B}" name="Roll No"/>
     <tableColumn id="2" xr3:uid="{8AA466D1-E11F-4916-9D39-98595DA9EC44}" name="Name"/>
     <tableColumn id="3" xr3:uid="{DDCF7F64-66EB-44A0-9F8F-114B7E458AF7}" name="Marks"/>
     <tableColumn id="4" xr3:uid="{37185CD3-B0CF-4A69-985F-3B3920FCA87E}" name="City"/>
-    <tableColumn id="5" xr3:uid="{37AE3DF9-4CBA-4A3F-A87D-31BC5F9E22E6}" name="Grade"/>
+    <tableColumn id="5" xr3:uid="{37AE3DF9-4CBA-4A3F-A87D-31BC5F9E22E6}" name="Result" dataDxfId="3">
+      <calculatedColumnFormula>IF(Table1[[#This Row],[Marks]]&gt;=40,"Pass","Fail")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{EA2F3D91-D920-463C-B54E-953C6D49CBF3}" name="Grade" dataDxfId="2">
+      <calculatedColumnFormula>IF(Table1[[#This Row],[Marks]]&gt;90,"A",IF(Table1[[#This Row],[Marks]]&gt;80,"B",IF(Table1[[#This Row],[Marks]]&gt;60,"C",IF(Table1[[#This Row],[Marks]]&gt;50,"D","F"))))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="7" xr3:uid="{62B22A3C-95D6-4E3B-8BA3-2B9B0D1A11C2}" name="And" dataDxfId="1">
+      <calculatedColumnFormula>AND(Table1[[#This Row],[Marks]]&gt;80,Table1[[#This Row],[City]]="Mumbai")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="8" xr3:uid="{BE70939C-AF73-4C6C-AF2C-1BF9B0DFECF3}" name="0r" dataDxfId="0">
+      <calculatedColumnFormula>OR(Table1[[#This Row],[Marks]]&gt;80,Table1[[#This Row],[City]]="Mumbai")</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -587,111 +628,111 @@
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="E2" s="1" t="s">
+      <c r="C2" s="4"/>
+      <c r="E2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="1"/>
-      <c r="H2" s="1" t="s">
+      <c r="F2" s="4"/>
+      <c r="H2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="1"/>
-      <c r="K2" s="1" t="s">
+      <c r="I2" s="4"/>
+      <c r="K2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="L2" s="1"/>
-      <c r="N2" s="1" t="s">
+      <c r="L2" s="4"/>
+      <c r="N2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="O2" s="1"/>
-      <c r="Q2" s="1" t="s">
+      <c r="O2" s="4"/>
+      <c r="Q2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="R2" s="1"/>
+      <c r="R2" s="4"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="B3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="2">
+      <c r="B3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="1">
         <f>LEN(B3)</f>
         <v>6</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="F3" s="2" t="str">
+      <c r="F3" s="1" t="str">
         <f>TRIM(E3)</f>
         <v>shashi</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="L3" s="2" t="str">
+      <c r="L3" s="1" t="str">
         <f>LEFT(K3,3)</f>
         <v>sha</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="N3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="O3" s="2" t="str">
+      <c r="O3" s="1" t="str">
         <f>RIGHT(N3,3)</f>
         <v>shi</v>
       </c>
-      <c r="Q3" s="2" t="s">
+      <c r="Q3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="R3" s="2" t="str">
+      <c r="R3" s="1" t="str">
         <f>MID(Q3,2,3)</f>
         <v>has</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <f>LEN(E3)</f>
         <v>9</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F4" s="1">
         <f>LEN(F3)</f>
         <v>6</v>
       </c>
-      <c r="H4" s="1" t="str">
+      <c r="H4" s="4" t="str">
         <f>_xlfn.CONCAT(H3,I3)</f>
         <v>raj patil</v>
       </c>
-      <c r="I4" s="1"/>
+      <c r="I4" s="4"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="1"/>
-      <c r="E6" s="1" t="s">
+      <c r="C6" s="4"/>
+      <c r="E6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="1"/>
+      <c r="F6" s="4"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="2" t="str">
+      <c r="C7" s="1" t="str">
         <f>UPPER(B7)</f>
         <v>SHASHI</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F7" s="2" t="str">
+      <c r="F7" s="1" t="str">
         <f>LOWER(E7)</f>
         <v>shashi</v>
       </c>
@@ -729,25 +770,25 @@
       <c r="C4" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <f ca="1">TODAY()</f>
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="5" spans="3:6" x14ac:dyDescent="0.3">
       <c r="C5" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="3">
         <f ca="1">NOW()</f>
-        <v>46303.86516828704</v>
+        <v>46304.822819328707</v>
       </c>
     </row>
     <row r="6" spans="3:6" x14ac:dyDescent="0.3">
       <c r="C6" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="2">
         <f>DATE(2029,12,23)</f>
         <v>47475</v>
       </c>
@@ -783,7 +824,7 @@
       </c>
       <c r="D9">
         <f ca="1">WEEKDAY(D4)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="3:6" x14ac:dyDescent="0.3">
@@ -811,13 +852,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC80CE97-5069-4B2C-852A-A81206AF3003}">
-  <dimension ref="C4:L14"/>
+  <dimension ref="C4:P17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="11" max="11" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="3:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C4" t="s">
         <v>37</v>
       </c>
@@ -831,17 +872,26 @@
         <v>40</v>
       </c>
       <c r="G4" t="s">
+        <v>50</v>
+      </c>
+      <c r="H4" t="s">
         <v>41</v>
       </c>
-      <c r="K4" t="s">
+      <c r="I4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J4" t="s">
+        <v>52</v>
+      </c>
+      <c r="O4" t="s">
         <v>42</v>
       </c>
-      <c r="L4">
+      <c r="P4">
         <f>SUM(Table1[Marks])</f>
-        <v>708</v>
-      </c>
-    </row>
-    <row r="5" spans="3:12" x14ac:dyDescent="0.3">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="5" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C5">
         <v>11</v>
       </c>
@@ -854,15 +904,31 @@
       <c r="F5" t="s">
         <v>33</v>
       </c>
-      <c r="K5" t="s">
+      <c r="G5" t="str">
+        <f>IF(Table1[[#This Row],[Marks]]&gt;=40,"Pass","Fail")</f>
+        <v>Pass</v>
+      </c>
+      <c r="H5" t="str">
+        <f>IF(Table1[[#This Row],[Marks]]&gt;90,"A",IF(Table1[[#This Row],[Marks]]&gt;80,"B",IF(Table1[[#This Row],[Marks]]&gt;60,"C",IF(Table1[[#This Row],[Marks]]&gt;50,"D","F"))))</f>
+        <v>D</v>
+      </c>
+      <c r="I5" t="b">
+        <f>AND(Table1[[#This Row],[Marks]]&gt;80,Table1[[#This Row],[City]]="Mumbai")</f>
+        <v>0</v>
+      </c>
+      <c r="J5" s="5" t="b">
+        <f>OR(Table1[[#This Row],[Marks]]&gt;80,Table1[[#This Row],[City]]="Mumbai")</f>
+        <v>1</v>
+      </c>
+      <c r="O5" t="s">
         <v>43</v>
       </c>
-      <c r="L5">
+      <c r="P5">
         <f>SUMIF(Table1[City],"Mumbai",Table1[Marks])</f>
         <v>201</v>
       </c>
     </row>
-    <row r="6" spans="3:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C6">
         <v>12</v>
       </c>
@@ -875,15 +941,31 @@
       <c r="F6" t="s">
         <v>34</v>
       </c>
-      <c r="K6" t="s">
+      <c r="G6" t="str">
+        <f>IF(Table1[[#This Row],[Marks]]&gt;=40,"Pass","Fail")</f>
+        <v>Pass</v>
+      </c>
+      <c r="H6" t="str">
+        <f>IF(Table1[[#This Row],[Marks]]&gt;90,"A",IF(Table1[[#This Row],[Marks]]&gt;80,"B",IF(Table1[[#This Row],[Marks]]&gt;60,"C",IF(Table1[[#This Row],[Marks]]&gt;50,"D","F"))))</f>
+        <v>B</v>
+      </c>
+      <c r="I6" t="b">
+        <f>AND(Table1[[#This Row],[Marks]]&gt;80,Table1[[#This Row],[City]]="Mumbai")</f>
+        <v>0</v>
+      </c>
+      <c r="J6" s="5" t="b">
+        <f>OR(Table1[[#This Row],[Marks]]&gt;80,Table1[[#This Row],[City]]="Mumbai")</f>
+        <v>1</v>
+      </c>
+      <c r="O6" t="s">
         <v>44</v>
       </c>
-      <c r="L6">
+      <c r="P6">
         <f>SUMIFS(Table1[Marks],Table1[City],"Mumbai",Table1[Marks],"&gt;70")</f>
         <v>89</v>
       </c>
     </row>
-    <row r="7" spans="3:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C7">
         <v>13</v>
       </c>
@@ -896,15 +978,31 @@
       <c r="F7" t="s">
         <v>33</v>
       </c>
-      <c r="K7" t="s">
+      <c r="G7" t="str">
+        <f>IF(Table1[[#This Row],[Marks]]&gt;=40,"Pass","Fail")</f>
+        <v>Pass</v>
+      </c>
+      <c r="H7" t="str">
+        <f>IF(Table1[[#This Row],[Marks]]&gt;90,"A",IF(Table1[[#This Row],[Marks]]&gt;80,"B",IF(Table1[[#This Row],[Marks]]&gt;60,"C",IF(Table1[[#This Row],[Marks]]&gt;50,"D","F"))))</f>
+        <v>B</v>
+      </c>
+      <c r="I7" t="b">
+        <f>AND(Table1[[#This Row],[Marks]]&gt;80,Table1[[#This Row],[City]]="Mumbai")</f>
+        <v>1</v>
+      </c>
+      <c r="J7" s="5" t="b">
+        <f>OR(Table1[[#This Row],[Marks]]&gt;80,Table1[[#This Row],[City]]="Mumbai")</f>
+        <v>1</v>
+      </c>
+      <c r="O7" t="s">
         <v>45</v>
       </c>
-      <c r="L7">
+      <c r="P7">
         <f>AVERAGE(Table1[Marks])</f>
-        <v>78.666666666666671</v>
-      </c>
-    </row>
-    <row r="8" spans="3:12" x14ac:dyDescent="0.3">
+        <v>72.444444444444443</v>
+      </c>
+    </row>
+    <row r="8" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C8">
         <v>14</v>
       </c>
@@ -917,15 +1015,31 @@
       <c r="F8" t="s">
         <v>35</v>
       </c>
-      <c r="K8" t="s">
+      <c r="G8" t="str">
+        <f>IF(Table1[[#This Row],[Marks]]&gt;=40,"Pass","Fail")</f>
+        <v>Pass</v>
+      </c>
+      <c r="H8" t="str">
+        <f>IF(Table1[[#This Row],[Marks]]&gt;90,"A",IF(Table1[[#This Row],[Marks]]&gt;80,"B",IF(Table1[[#This Row],[Marks]]&gt;60,"C",IF(Table1[[#This Row],[Marks]]&gt;50,"D","F"))))</f>
+        <v>C</v>
+      </c>
+      <c r="I8" t="b">
+        <f>AND(Table1[[#This Row],[Marks]]&gt;80,Table1[[#This Row],[City]]="Mumbai")</f>
+        <v>0</v>
+      </c>
+      <c r="J8" s="5" t="b">
+        <f>OR(Table1[[#This Row],[Marks]]&gt;80,Table1[[#This Row],[City]]="Mumbai")</f>
+        <v>0</v>
+      </c>
+      <c r="O8" t="s">
         <v>46</v>
       </c>
-      <c r="L8">
+      <c r="P8">
         <f>AVERAGEIF(Table1[Marks],"&gt;70")</f>
-        <v>85.142857142857139</v>
-      </c>
-    </row>
-    <row r="9" spans="3:12" x14ac:dyDescent="0.3">
+        <v>84.333333333333329</v>
+      </c>
+    </row>
+    <row r="9" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C9">
         <v>15</v>
       </c>
@@ -933,20 +1047,36 @@
         <v>28</v>
       </c>
       <c r="E9">
-        <v>90</v>
+        <v>34</v>
       </c>
       <c r="F9" t="s">
         <v>36</v>
       </c>
-      <c r="K9" t="s">
+      <c r="G9" t="str">
+        <f>IF(Table1[[#This Row],[Marks]]&gt;=40,"Pass","Fail")</f>
+        <v>Fail</v>
+      </c>
+      <c r="H9" t="str">
+        <f>IF(Table1[[#This Row],[Marks]]&gt;90,"A",IF(Table1[[#This Row],[Marks]]&gt;80,"B",IF(Table1[[#This Row],[Marks]]&gt;60,"C",IF(Table1[[#This Row],[Marks]]&gt;50,"D","F"))))</f>
+        <v>F</v>
+      </c>
+      <c r="I9" t="b">
+        <f>AND(Table1[[#This Row],[Marks]]&gt;80,Table1[[#This Row],[City]]="Mumbai")</f>
+        <v>0</v>
+      </c>
+      <c r="J9" s="5" t="b">
+        <f>OR(Table1[[#This Row],[Marks]]&gt;80,Table1[[#This Row],[City]]="Mumbai")</f>
+        <v>0</v>
+      </c>
+      <c r="O9" t="s">
         <v>47</v>
       </c>
-      <c r="L9">
+      <c r="P9">
         <f>COUNT(Table1[Roll No])</f>
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="3:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C10">
         <v>16</v>
       </c>
@@ -959,15 +1089,31 @@
       <c r="F10" t="s">
         <v>35</v>
       </c>
-      <c r="K10" t="s">
+      <c r="G10" t="str">
+        <f>IF(Table1[[#This Row],[Marks]]&gt;=40,"Pass","Fail")</f>
+        <v>Pass</v>
+      </c>
+      <c r="H10" t="str">
+        <f>IF(Table1[[#This Row],[Marks]]&gt;90,"A",IF(Table1[[#This Row],[Marks]]&gt;80,"B",IF(Table1[[#This Row],[Marks]]&gt;60,"C",IF(Table1[[#This Row],[Marks]]&gt;50,"D","F"))))</f>
+        <v>A</v>
+      </c>
+      <c r="I10" t="b">
+        <f>AND(Table1[[#This Row],[Marks]]&gt;80,Table1[[#This Row],[City]]="Mumbai")</f>
+        <v>0</v>
+      </c>
+      <c r="J10" s="5" t="b">
+        <f>OR(Table1[[#This Row],[Marks]]&gt;80,Table1[[#This Row],[City]]="Mumbai")</f>
+        <v>1</v>
+      </c>
+      <c r="O10" t="s">
         <v>48</v>
       </c>
-      <c r="L10">
+      <c r="P10">
         <f>COUNTA(Table1[Roll No])</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="3:12" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C11">
         <v>17</v>
       </c>
@@ -980,15 +1126,31 @@
       <c r="F11" t="s">
         <v>34</v>
       </c>
-      <c r="K11" t="s">
-        <v>50</v>
-      </c>
-      <c r="L11">
-        <f>COUNTBLANK(C5:C15)</f>
+      <c r="G11" t="str">
+        <f>IF(Table1[[#This Row],[Marks]]&gt;=40,"Pass","Fail")</f>
+        <v>Pass</v>
+      </c>
+      <c r="H11" t="str">
+        <f>IF(Table1[[#This Row],[Marks]]&gt;90,"A",IF(Table1[[#This Row],[Marks]]&gt;80,"B",IF(Table1[[#This Row],[Marks]]&gt;60,"C",IF(Table1[[#This Row],[Marks]]&gt;50,"D","F"))))</f>
+        <v>C</v>
+      </c>
+      <c r="I11" t="b">
+        <f>AND(Table1[[#This Row],[Marks]]&gt;80,Table1[[#This Row],[City]]="Mumbai")</f>
+        <v>0</v>
+      </c>
+      <c r="J11" s="5" t="b">
+        <f>OR(Table1[[#This Row],[Marks]]&gt;80,Table1[[#This Row],[City]]="Mumbai")</f>
+        <v>0</v>
+      </c>
+      <c r="O11" t="s">
+        <v>49</v>
+      </c>
+      <c r="P11">
+        <f>COUNTBLANK(C5:C14)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="3:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C12">
         <v>18</v>
       </c>
@@ -1001,8 +1163,24 @@
       <c r="F12" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="13" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="G12" t="str">
+        <f>IF(Table1[[#This Row],[Marks]]&gt;=40,"Pass","Fail")</f>
+        <v>Pass</v>
+      </c>
+      <c r="H12" t="str">
+        <f>IF(Table1[[#This Row],[Marks]]&gt;90,"A",IF(Table1[[#This Row],[Marks]]&gt;80,"B",IF(Table1[[#This Row],[Marks]]&gt;60,"C",IF(Table1[[#This Row],[Marks]]&gt;50,"D","F"))))</f>
+        <v>D</v>
+      </c>
+      <c r="I12" t="b">
+        <f>AND(Table1[[#This Row],[Marks]]&gt;80,Table1[[#This Row],[City]]="Mumbai")</f>
+        <v>0</v>
+      </c>
+      <c r="J12" s="5" t="b">
+        <f>OR(Table1[[#This Row],[Marks]]&gt;80,Table1[[#This Row],[City]]="Mumbai")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C13">
         <v>19</v>
       </c>
@@ -1015,13 +1193,43 @@
       <c r="F13" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="14" spans="3:12" x14ac:dyDescent="0.3">
-      <c r="C14" t="s">
-        <v>49</v>
+      <c r="G13" t="str">
+        <f>IF(Table1[[#This Row],[Marks]]&gt;=40,"Pass","Fail")</f>
+        <v>Pass</v>
+      </c>
+      <c r="H13" t="str">
+        <f>IF(Table1[[#This Row],[Marks]]&gt;90,"A",IF(Table1[[#This Row],[Marks]]&gt;80,"B",IF(Table1[[#This Row],[Marks]]&gt;60,"C",IF(Table1[[#This Row],[Marks]]&gt;50,"D","F"))))</f>
+        <v>C</v>
+      </c>
+      <c r="I13" t="b">
+        <f>AND(Table1[[#This Row],[Marks]]&gt;80,Table1[[#This Row],[City]]="Mumbai")</f>
+        <v>0</v>
+      </c>
+      <c r="J13" s="5" t="b">
+        <f>OR(Table1[[#This Row],[Marks]]&gt;80,Table1[[#This Row],[City]]="Mumbai")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="3:16" x14ac:dyDescent="0.3">
+      <c r="C16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D16" s="6"/>
+    </row>
+    <row r="17" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C17" t="e">
+        <f>6/0</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D17">
+        <f>IFERROR(4/0,0)</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C16:D16"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>